<commit_message>
Changes to Torre_Rsina params
</commit_message>
<xml_diff>
--- a/Torre_Orsina/Parameters/Options_and_NoVegParams.xlsx
+++ b/Torre_Orsina/Parameters/Options_and_NoVegParams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\group\pelligrp\Project_folders\MountainWater\Tethys_Chloris\Workflow_dev\Scripts\Cat\TeC_Source_Code\Torre_Orsina\Parameters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88498B87-3A30-4EF2-A1C9-8703E5EF1C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F975AD4F-BB72-4B15-BF4E-4E51718834E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-5475" windowWidth="29040" windowHeight="17520" xr2:uid="{1C5B3D2E-5EDA-40D4-886E-AB020D607408}"/>
   </bookViews>
@@ -1813,7 +1813,7 @@
         <v>106</v>
       </c>
       <c r="G33" s="8">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>39</v>

</xml_diff>